<commit_message>
Add Contenidos_Consultados_v2.py with improved PBI replication
- Filtrado en 2 capas: patrones dinámicos (CONTAINS) + lista manual
- Agrupación por prefijo (RulenameUnique) con max por día
- Agrupación especial TUR00CUX02: solo la de mayor valor (nueva política)
- Nombres amigables para el top 10 y Excel detallado
- Exclusión de miBA como patrón en Capa 1
- Regenerados outputs enero y febrero 2026

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Contenidos_Consultados/output/contenidos_consultados_enero_2026.xlsx
+++ b/Contenidos_Consultados/output/contenidos_consultados_enero_2026.xlsx
@@ -55,10 +55,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,7 +432,7 @@
   <cols>
     <col width="35" customWidth="1" min="2" max="2"/>
     <col width="50" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -569,16 +572,27 @@
     <row r="11">
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>contenidos mas consultados</t>
+          <t>Contenidos más consultados</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Q Contenidos con más interacciones en el mes (Top 20)</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="n">
-        <v>5430</v>
+          <t>Q Contenidos con más interacciones en el mes</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>1- Confirmación Turnos Salud: (491.135)
+2- Infracciones: (160.845)
+3- Turnos Salud: (132.737)
+4- Trámites Vehículos SAP: (118.479)
+5- Mis profesionales: (109.130)
+6- Licencias: (82.617)
+7- Hospitales: (81.726)
+8- Licencia prorroga  &gt; Consultar: (73.806)
+9- Trámites SAP: (70.865)
+10- MO05CUX01 &gt; Tiene que renovar: (55.176)</t>
+        </is>
       </c>
     </row>
     <row r="12">

</xml_diff>

<commit_message>
Regenerar outputs enero 2026 con exclusiones actualizadas
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Contenidos_Consultados/output/contenidos_consultados_enero_2026.xlsx
+++ b/Contenidos_Consultados/output/contenidos_consultados_enero_2026.xlsx
@@ -589,9 +589,9 @@
 5- Mis profesionales: (109.130)
 6- Licencias: (82.617)
 7- Hospitales: (81.726)
-8- Licencia prorroga  &gt; Consultar: (73.806)
-9- Trámites SAP: (70.865)
-10- MO05CUX01 &gt; Tiene que renovar: (55.176)</t>
+8- Trámites SAP: (70.865)
+9- Buscar donde está permitido estacionar: (40.441)
+10- Permitido estacionar por dirección: (23.309)</t>
         </is>
       </c>
     </row>

</xml_diff>